<commit_message>
before adding RTO logic in Print_tshirt_inventory while print and merch deductions
</commit_message>
<xml_diff>
--- a/Employee Inventory Tracker.xlsx
+++ b/Employee Inventory Tracker.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\expense tracker\ajio\Return Automation\ajio-return-sync\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC5BD1C-B368-4B3C-BF02-DAE42265828B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D964560-AFA1-43E9-B8F9-2D24111C9F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WeeklyStockCount" sheetId="1" r:id="rId1"/>
-    <sheet name="UpdateInventory" sheetId="2" r:id="rId2"/>
-    <sheet name="ReviewWeeklyStockUpdates" sheetId="3" r:id="rId3"/>
+    <sheet name="ReviewWeeklyStockUpdates" sheetId="3" r:id="rId2"/>
+    <sheet name="UpdateInventory" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="66">
   <si>
     <t>Slot</t>
   </si>
@@ -229,7 +229,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-mmmm\-yyyy"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -331,6 +331,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="26">
     <fill>
@@ -496,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -540,6 +547,7 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1463,956 +1471,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28.77734375" customWidth="1"/>
-    <col min="2" max="2" width="15.21875" customWidth="1"/>
-    <col min="4" max="4" width="5" customWidth="1"/>
-    <col min="5" max="5" width="5.44140625" customWidth="1"/>
-    <col min="6" max="6" width="5.109375" customWidth="1"/>
-    <col min="7" max="7" width="6" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-      <c r="G12" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0</v>
-      </c>
-      <c r="G13" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0</v>
-      </c>
-      <c r="F14" s="1">
-        <v>0</v>
-      </c>
-      <c r="G14" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="1">
-        <v>0</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
-      <c r="F15" s="1">
-        <v>0</v>
-      </c>
-      <c r="G15" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="1">
-        <v>0</v>
-      </c>
-      <c r="E16" s="1">
-        <v>0</v>
-      </c>
-      <c r="F16" s="1">
-        <v>0</v>
-      </c>
-      <c r="G16" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="1">
-        <v>0</v>
-      </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
-      <c r="F17" s="1">
-        <v>0</v>
-      </c>
-      <c r="G17" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="1">
-        <v>0</v>
-      </c>
-      <c r="E18" s="1">
-        <v>0</v>
-      </c>
-      <c r="F18" s="1">
-        <v>0</v>
-      </c>
-      <c r="G18" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="1">
-        <v>0</v>
-      </c>
-      <c r="E19" s="1">
-        <v>0</v>
-      </c>
-      <c r="F19" s="1">
-        <v>0</v>
-      </c>
-      <c r="G19" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="1">
-        <v>0</v>
-      </c>
-      <c r="E20" s="1">
-        <v>0</v>
-      </c>
-      <c r="F20" s="1">
-        <v>0</v>
-      </c>
-      <c r="G20" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="1">
-        <v>0</v>
-      </c>
-      <c r="E21" s="1">
-        <v>0</v>
-      </c>
-      <c r="F21" s="1">
-        <v>0</v>
-      </c>
-      <c r="G21" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="1">
-        <v>0</v>
-      </c>
-      <c r="E22" s="1">
-        <v>0</v>
-      </c>
-      <c r="F22" s="1">
-        <v>0</v>
-      </c>
-      <c r="G22" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="1">
-        <v>0</v>
-      </c>
-      <c r="E23" s="1">
-        <v>0</v>
-      </c>
-      <c r="F23" s="1">
-        <v>0</v>
-      </c>
-      <c r="G23" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1">
-        <v>0</v>
-      </c>
-      <c r="F24" s="1">
-        <v>0</v>
-      </c>
-      <c r="G24" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="1">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1">
-        <v>0</v>
-      </c>
-      <c r="G25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="1">
-        <v>0</v>
-      </c>
-      <c r="E26" s="1">
-        <v>0</v>
-      </c>
-      <c r="F26" s="1">
-        <v>0</v>
-      </c>
-      <c r="G26" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0</v>
-      </c>
-      <c r="E27" s="1">
-        <v>0</v>
-      </c>
-      <c r="F27" s="1">
-        <v>0</v>
-      </c>
-      <c r="G27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="1">
-        <v>0</v>
-      </c>
-      <c r="E28" s="1">
-        <v>0</v>
-      </c>
-      <c r="F28" s="1">
-        <v>0</v>
-      </c>
-      <c r="G28" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D29" s="1">
-        <v>0</v>
-      </c>
-      <c r="E29" s="1">
-        <v>0</v>
-      </c>
-      <c r="F29" s="1">
-        <v>0</v>
-      </c>
-      <c r="G29" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="1">
-        <v>0</v>
-      </c>
-      <c r="E30" s="1">
-        <v>0</v>
-      </c>
-      <c r="F30" s="1">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D31" s="1">
-        <v>0</v>
-      </c>
-      <c r="E31" s="1">
-        <v>0</v>
-      </c>
-      <c r="F31" s="1">
-        <v>0</v>
-      </c>
-      <c r="G31" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="33" t="s">
-        <v>44</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="1">
-        <v>0</v>
-      </c>
-      <c r="E32" s="1">
-        <v>0</v>
-      </c>
-      <c r="F32" s="1">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D33" s="1">
-        <v>0</v>
-      </c>
-      <c r="E33" s="1">
-        <v>0</v>
-      </c>
-      <c r="F33" s="1">
-        <v>0</v>
-      </c>
-      <c r="G33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="1">
-        <v>0</v>
-      </c>
-      <c r="E34" s="1">
-        <v>0</v>
-      </c>
-      <c r="F34" s="1">
-        <v>0</v>
-      </c>
-      <c r="G34" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A35" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D35" s="1">
-        <v>0</v>
-      </c>
-      <c r="E35" s="1">
-        <v>0</v>
-      </c>
-      <c r="F35" s="1">
-        <v>0</v>
-      </c>
-      <c r="G35" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D36" s="1">
-        <v>0</v>
-      </c>
-      <c r="E36" s="1">
-        <v>0</v>
-      </c>
-      <c r="F36" s="1">
-        <v>0</v>
-      </c>
-      <c r="G36" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A37" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="1">
-        <v>0</v>
-      </c>
-      <c r="E37" s="1">
-        <v>0</v>
-      </c>
-      <c r="F37" s="1">
-        <v>0</v>
-      </c>
-      <c r="G37" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0</v>
-      </c>
-      <c r="E38" s="1">
-        <v>0</v>
-      </c>
-      <c r="F38" s="1">
-        <v>0</v>
-      </c>
-      <c r="G38" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D39" s="1">
-        <v>0</v>
-      </c>
-      <c r="E39" s="1">
-        <v>0</v>
-      </c>
-      <c r="F39" s="1">
-        <v>0</v>
-      </c>
-      <c r="G39" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="B40" s="42" t="s">
-        <v>58</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="1">
-        <v>0</v>
-      </c>
-      <c r="E40" s="1">
-        <v>0</v>
-      </c>
-      <c r="F40" s="1">
-        <v>0</v>
-      </c>
-      <c r="G40" s="1">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C40" xr:uid="{00000000-0002-0000-0100-000000000000}">
-      <formula1>"Select,Add,Reduce,Replace"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FDD73D1-8BD3-4B0D-974C-13F5D88714AB}">
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -2442,4 +1505,954 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:K40"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.77734375" customWidth="1"/>
+    <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="4" max="4" width="5" customWidth="1"/>
+    <col min="5" max="5" width="5.44140625" customWidth="1"/>
+    <col min="6" max="6" width="5.109375" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="43" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0</v>
+      </c>
+      <c r="G22" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0</v>
+      </c>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0</v>
+      </c>
+      <c r="F28" s="1">
+        <v>0</v>
+      </c>
+      <c r="G28" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0</v>
+      </c>
+      <c r="E29" s="1">
+        <v>0</v>
+      </c>
+      <c r="F29" s="1">
+        <v>0</v>
+      </c>
+      <c r="G29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="1">
+        <v>0</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1">
+        <v>0</v>
+      </c>
+      <c r="G31" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0</v>
+      </c>
+      <c r="E33" s="1">
+        <v>0</v>
+      </c>
+      <c r="F33" s="1">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1">
+        <v>0</v>
+      </c>
+      <c r="F34" s="1">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1">
+        <v>0</v>
+      </c>
+      <c r="G35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1">
+        <v>0</v>
+      </c>
+      <c r="G36" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A37" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1">
+        <v>0</v>
+      </c>
+      <c r="F37" s="1">
+        <v>0</v>
+      </c>
+      <c r="G37" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1">
+        <v>0</v>
+      </c>
+      <c r="G38" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="1">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1">
+        <v>0</v>
+      </c>
+      <c r="F39" s="1">
+        <v>0</v>
+      </c>
+      <c r="G39" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1">
+        <v>0</v>
+      </c>
+      <c r="F40" s="1">
+        <v>0</v>
+      </c>
+      <c r="G40" s="1">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C40" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"Select,Add,Reduce,Replace"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>